<commit_message>
Update April 2026 PUN PSV indices
</commit_message>
<xml_diff>
--- a/indici_pun_psv_2025_2026.xlsx
+++ b/indici_pun_psv_2025_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/silviofornaro/Desktop/EnergiaSolidaleLast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038405A5-68CA-CB45-A540-AF499CE9B090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07DD7685-B50A-C145-8095-12054263105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36640" yWindow="5840" windowWidth="30380" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30980" yWindow="1440" windowWidth="30380" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indici" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <r>
       <rPr>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>mese</t>
+  </si>
+  <si>
+    <t>2026-04</t>
   </si>
 </sst>
 </file>
@@ -517,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="69.3984375" customWidth="1"/>
@@ -536,173 +539,184 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" ht="41" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.12200999999999999</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.49232500000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="30.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B3" s="4">
         <v>0.14500666666666667</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C3" s="4">
         <v>0.55769999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="3" t="s">
+    <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B4" s="4">
         <v>0.11580666666666667</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C4" s="4">
         <v>0.377</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B5" s="4">
         <v>0.13639666666666667</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C5" s="4">
         <v>0.40400000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B6" s="4">
         <v>0.11813</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C6" s="4">
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B7" s="4">
         <v>0.11970666666666667</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C7" s="4">
         <v>0.34899999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B8" s="4">
         <v>0.11302333333333332</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C8" s="4">
         <v>0.35399999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B9" s="4">
         <v>0.11080000000000001</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C9" s="4">
         <v>0.373</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="3" t="s">
+    <row r="10" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B10" s="4">
         <v>0.10986333333333333</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C10" s="4">
         <v>0.38100000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B11" s="4">
         <v>0.11484</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C11" s="4">
         <v>0.39200000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="3" t="s">
+    <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B12" s="4">
         <v>0.11448333333333334</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C12" s="4">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="3" t="s">
+    <row r="13" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B13" s="4">
         <v>9.5613333333333342E-2</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C13" s="4">
         <v>0.40300000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="3" t="s">
+    <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B14" s="4">
         <v>0.10198999999999998</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C14" s="4">
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B15" s="4">
         <v>0.12273000000000001</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C15" s="4">
         <v>0.45500000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="3" t="s">
+    <row r="16" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B16" s="4">
         <v>0.15216666666666667</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C16" s="4">
         <v>0.56599999999999995</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="5" t="s">
+    <row r="17" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B17" s="4">
         <v>0.14615666666666666</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.15">
-      <c r="B17" s="2"/>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="B18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add invite-only Illumia customer area
</commit_message>
<xml_diff>
--- a/indici_pun_psv_2025_2026.xlsx
+++ b/indici_pun_psv_2025_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/silviofornaro/Desktop/EnergiaSolidaleLast/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/EnergiaSolidaleLast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07DD7685-B50A-C145-8095-12054263105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BC1A3D-A8C2-0F41-88AA-D0DD17685961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30980" yWindow="1440" windowWidth="30380" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indici" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <r>
       <rPr>
@@ -102,6 +102,9 @@
   <si>
     <t>2026-04</t>
   </si>
+  <si>
+    <t>2006-05</t>
+  </si>
 </sst>
 </file>
 
@@ -110,7 +113,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -153,6 +156,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF515151"/>
+      <name val="Inherit"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -194,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -215,6 +223,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,15 +531,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="69.3984375" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="27.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="41" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:8" ht="41" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>18</v>
       </c>
@@ -539,184 +550,198 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="41" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:8" ht="41" customHeight="1">
       <c r="A2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.119807</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.50961999999999996</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="41" customHeight="1">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B3" s="4">
         <v>0.12200999999999999</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C3" s="4">
         <v>0.49232500000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="30.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="3" t="s">
+    <row r="4" spans="1:8" ht="30.25" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B4" s="4">
         <v>0.14500666666666667</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C4" s="4">
         <v>0.55769999999999997</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="3" t="s">
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" ht="32" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B5" s="4">
         <v>0.11580666666666667</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C5" s="4">
         <v>0.377</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:8" ht="32.5" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B6" s="4">
         <v>0.13639666666666667</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C6" s="4">
         <v>0.40400000000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B7" s="4">
         <v>0.11813</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C7" s="4">
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:8" ht="32" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B8" s="4">
         <v>0.11970666666666667</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C8" s="4">
         <v>0.34899999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B9" s="4">
         <v>0.11302333333333332</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C9" s="4">
         <v>0.35399999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="3" t="s">
+    <row r="10" spans="1:8" ht="32" customHeight="1">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B10" s="4">
         <v>0.11080000000000001</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C10" s="4">
         <v>0.373</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B11" s="4">
         <v>0.10986333333333333</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C11" s="4">
         <v>0.38100000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="3" t="s">
+    <row r="12" spans="1:8" ht="32.5" customHeight="1">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B12" s="4">
         <v>0.11484</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C12" s="4">
         <v>0.39200000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="3" t="s">
+    <row r="13" spans="1:8" ht="32" customHeight="1">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B13" s="4">
         <v>0.11448333333333334</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C13" s="4">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="3" t="s">
+    <row r="14" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B14" s="4">
         <v>9.5613333333333342E-2</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C14" s="4">
         <v>0.40300000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:8" ht="32" customHeight="1">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B15" s="4">
         <v>0.10198999999999998</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C15" s="4">
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="3" t="s">
+    <row r="16" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B16" s="4">
         <v>0.12273000000000001</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C16" s="4">
         <v>0.45500000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="3" t="s">
+    <row r="17" spans="1:3" ht="32.5" customHeight="1">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B17" s="4">
         <v>0.15216666666666667</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C17" s="4">
         <v>0.56599999999999995</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="5" t="s">
+    <row r="18" spans="1:3" ht="23.25" customHeight="1">
+      <c r="A18" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B18" s="4">
         <v>0.14615666666666666</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
-      <c r="B18" s="2"/>
+    <row r="19" spans="1:3">
+      <c r="B19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>